<commit_message>
Regenerate workbook with segment PP&E and update verification
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SpaceX_Cursor_Pro_Forma_Model.xlsx
+++ b/SpaceX_Cursor_Pro_Forma_Model.xlsx
@@ -698,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1076,332 +1076,397 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex % of combined revenue</t>
+          <t xml:space="preserve">  Space — capex % of segment revenue</t>
         </is>
       </c>
       <c r="C21" s="12" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D21" s="12" t="n">
         <v>0.26</v>
       </c>
-      <c r="D21" s="12" t="n">
-        <v>0.23</v>
-      </c>
       <c r="E21" s="12" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="G21" s="12" t="n">
-        <v>0.175</v>
+        <v>0.2</v>
       </c>
       <c r="H21" s="12" t="n">
-        <v>0.165</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Depreciation % of beginning net PP&amp;E</t>
+          <t xml:space="preserve">  Starlink — capex % of segment revenue</t>
         </is>
       </c>
       <c r="C22" s="12" t="n">
-        <v>0.09</v>
+        <v>0.36</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>0.22</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A allocation — Space %</t>
+          <t xml:space="preserve">  xAI-Cursor — capex % of segment revenue</t>
         </is>
       </c>
       <c r="C23" s="12" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E23" s="12" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F23" s="12" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G23" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H23" s="12" t="n">
+        <v>0.18</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A allocation — Starlink %</t>
+          <t xml:space="preserve">  Space — depreciation % of beginning PP&amp;E</t>
         </is>
       </c>
       <c r="C24" s="12" t="n">
-        <v>0.5</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A allocation — xAI-Cursor %</t>
+          <t xml:space="preserve">  Starlink — depreciation % of beginning PP&amp;E</t>
         </is>
       </c>
       <c r="C25" s="12" t="n">
-        <v>0.2</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stock-based comp % of revenue</t>
+          <t xml:space="preserve">  xAI-Cursor — depreciation % of beginning PP&amp;E</t>
         </is>
       </c>
       <c r="C26" s="12" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="D26" s="12" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="E26" s="12" t="n">
-        <v>0.055</v>
-      </c>
-      <c r="F26" s="12" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G26" s="12" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="H26" s="12" t="n">
-        <v>0.04</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net new long-term debt ($M)</t>
+          <t xml:space="preserve">  Space — opening net PP&amp;E ($M)</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="11" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E27" s="11" t="n">
-        <v>2000</v>
-      </c>
-      <c r="F27" s="11" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G27" s="11" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H27" s="11" t="n">
-        <v>1000</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Spectrum obligation repayment ($M)</t>
+          <t xml:space="preserve">  xAI-Cursor — opening net PP&amp;E ($M)</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="11" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="E28" s="11" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="F28" s="11" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="G28" s="11" t="n">
-        <v>-2000</v>
-      </c>
-      <c r="H28" s="11" t="n">
-        <v>-2000</v>
+        <v>3300</v>
+      </c>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>Starlink opening = total − Space − xAI-Cursor</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Primary equity issuance / IPO proceeds ($M)</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="11" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E29" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="13" t="inlineStr">
-        <is>
-          <t>SpaceX June-2026 IPO</t>
-        </is>
+          <t xml:space="preserve">  Stock-based comp % of revenue</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="F29" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>0.04</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Interest rate on debt &amp; spectrum obligation</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="n">
-        <v>0.065</v>
+          <t xml:space="preserve">  Net new long-term debt ($M)</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <v>1500</v>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H30" s="11" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Interest income rate on cash</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="n">
-        <v>0.04</v>
+          <t xml:space="preserve">  Spectrum obligation repayment ($M)</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="E31" s="11" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="F31" s="11" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="G31" s="11" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="H31" s="11" t="n">
+        <v>-2000</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Statutory tax rate</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="n">
-        <v>0.21</v>
+          <t xml:space="preserve">  Primary equity issuance / IPO proceeds ($M)</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="11" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="13" t="inlineStr">
+        <is>
+          <t>SpaceX June-2026 IPO</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Opening NOL carryforward, FY2025 ($M)</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="n">
-        <v>26000</v>
-      </c>
-      <c r="L33" s="13" t="inlineStr">
-        <is>
-          <t>SpaceX accumulated + Cursor</t>
-        </is>
+          <t xml:space="preserve">  Interest rate on debt &amp; spectrum obligation</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>0.065</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOL usage limit (% of taxable income)</t>
+          <t xml:space="preserve">  Interest income rate on cash</t>
         </is>
       </c>
       <c r="C34" s="12" t="n">
-        <v>0.8</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SpaceX shares pre-deal (M)</t>
-        </is>
-      </c>
-      <c r="C35" s="14" t="n">
-        <v>2000</v>
+          <t xml:space="preserve">  Statutory tax rate</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n">
+        <v>0.21</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SpaceX share price, deal pricing ($)</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="n">
-        <v>450</v>
+          <t xml:space="preserve">  Opening NOL carryforward, FY2025 ($M)</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>26000</v>
+      </c>
+      <c r="L36" s="13" t="inlineStr">
+        <is>
+          <t>SpaceX accumulated + Cursor</t>
+        </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>Working capital ratios (% of revenue)</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="n"/>
-      <c r="C37" s="9" t="n"/>
-      <c r="D37" s="9" t="n"/>
-      <c r="E37" s="9" t="n"/>
-      <c r="F37" s="9" t="n"/>
-      <c r="G37" s="9" t="n"/>
-      <c r="H37" s="9" t="n"/>
-      <c r="I37" s="9" t="n"/>
-      <c r="J37" s="9" t="n"/>
-      <c r="K37" s="9" t="n"/>
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOL usage limit (% of taxable income)</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts receivable (% of revenue)</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="n">
-        <v>0.1339</v>
+          <t xml:space="preserve">  SpaceX shares pre-deal (M)</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Inventory (% of revenue)</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="n">
-        <v>0.1499</v>
+          <t xml:space="preserve">  SpaceX share price, deal pricing ($)</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="n">
+        <v>450</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Prepaid &amp; other current assets (% of revenue)</t>
-        </is>
-      </c>
-      <c r="C40" s="12" t="n">
-        <v>0.0803</v>
-      </c>
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>Working capital ratios (% of revenue)</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="n"/>
+      <c r="C40" s="9" t="n"/>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="9" t="n"/>
+      <c r="F40" s="9" t="n"/>
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9" t="n"/>
+      <c r="I40" s="9" t="n"/>
+      <c r="J40" s="9" t="n"/>
+      <c r="K40" s="9" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accounts payable (% of revenue)</t>
+          <t xml:space="preserve">  Accounts receivable (% of revenue)</t>
         </is>
       </c>
       <c r="C41" s="12" t="n">
-        <v>0.1499</v>
+        <v>0.1339</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Accrued liabilities (% of revenue)</t>
+          <t xml:space="preserve">  Inventory (% of revenue)</t>
         </is>
       </c>
       <c r="C42" s="12" t="n">
-        <v>0.091</v>
+        <v>0.1499</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Deferred revenue, current (% of revenue)</t>
+          <t xml:space="preserve">  Prepaid &amp; other current assets (% of revenue)</t>
         </is>
       </c>
       <c r="C43" s="12" t="n">
-        <v>0.1499</v>
+        <v>0.0803</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Accounts payable (% of revenue)</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>0.1499</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Accrued liabilities (% of revenue)</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>0.091</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Deferred revenue, current (% of revenue)</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="n">
+        <v>0.1499</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Customer deposits &amp; advances (% of revenue)</t>
         </is>
       </c>
-      <c r="C44" s="12" t="n">
+      <c r="C47" s="12" t="n">
         <v>0.1017</v>
       </c>
     </row>
@@ -1875,7 +1940,7 @@
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  D&amp;A by capital-intensity weights; net interest &amp; tax allocated by revenue share.</t>
+          <t xml:space="preserve">  Segment D&amp;A from the PP&amp;E schedule; net interest &amp; tax allocated by revenue share.</t>
         </is>
       </c>
     </row>
@@ -1924,27 +1989,27 @@
         </is>
       </c>
       <c r="C21" s="16">
-        <f>-'Income Statement'!C16*'Assumptions'!C23</f>
+        <f>-'Schedules'!C7</f>
         <v/>
       </c>
       <c r="D21" s="16">
-        <f>-'Income Statement'!D16*'Assumptions'!C23</f>
+        <f>-'Schedules'!D7</f>
         <v/>
       </c>
       <c r="E21" s="16">
-        <f>-'Income Statement'!E16*'Assumptions'!C23</f>
+        <f>-'Schedules'!E7</f>
         <v/>
       </c>
       <c r="F21" s="16">
-        <f>-'Income Statement'!F16*'Assumptions'!C23</f>
+        <f>-'Schedules'!F7</f>
         <v/>
       </c>
       <c r="G21" s="16">
-        <f>-'Income Statement'!G16*'Assumptions'!C23</f>
+        <f>-'Schedules'!G7</f>
         <v/>
       </c>
       <c r="H21" s="16">
-        <f>-'Income Statement'!H16*'Assumptions'!C23</f>
+        <f>-'Schedules'!H7</f>
         <v/>
       </c>
     </row>
@@ -2204,27 +2269,27 @@
         </is>
       </c>
       <c r="C31" s="16">
-        <f>-'Income Statement'!C16*'Assumptions'!C24</f>
+        <f>-'Schedules'!C12</f>
         <v/>
       </c>
       <c r="D31" s="16">
-        <f>-'Income Statement'!D16*'Assumptions'!C24</f>
+        <f>-'Schedules'!D12</f>
         <v/>
       </c>
       <c r="E31" s="16">
-        <f>-'Income Statement'!E16*'Assumptions'!C24</f>
+        <f>-'Schedules'!E12</f>
         <v/>
       </c>
       <c r="F31" s="16">
-        <f>-'Income Statement'!F16*'Assumptions'!C24</f>
+        <f>-'Schedules'!F12</f>
         <v/>
       </c>
       <c r="G31" s="16">
-        <f>-'Income Statement'!G16*'Assumptions'!C24</f>
+        <f>-'Schedules'!G12</f>
         <v/>
       </c>
       <c r="H31" s="16">
-        <f>-'Income Statement'!H16*'Assumptions'!C24</f>
+        <f>-'Schedules'!H12</f>
         <v/>
       </c>
     </row>
@@ -2484,27 +2549,27 @@
         </is>
       </c>
       <c r="C41" s="16">
-        <f>-'Income Statement'!C16*'Assumptions'!C25</f>
+        <f>-'Schedules'!C17</f>
         <v/>
       </c>
       <c r="D41" s="16">
-        <f>-'Income Statement'!D16*'Assumptions'!C25</f>
+        <f>-'Schedules'!D17</f>
         <v/>
       </c>
       <c r="E41" s="16">
-        <f>-'Income Statement'!E16*'Assumptions'!C25</f>
+        <f>-'Schedules'!E17</f>
         <v/>
       </c>
       <c r="F41" s="16">
-        <f>-'Income Statement'!F16*'Assumptions'!C25</f>
+        <f>-'Schedules'!F17</f>
         <v/>
       </c>
       <c r="G41" s="16">
-        <f>-'Income Statement'!G16*'Assumptions'!C25</f>
+        <f>-'Schedules'!G17</f>
         <v/>
       </c>
       <c r="H41" s="16">
-        <f>-'Income Statement'!H16*'Assumptions'!C25</f>
+        <f>-'Schedules'!H17</f>
         <v/>
       </c>
     </row>
@@ -2863,7 +2928,7 @@
         </is>
       </c>
       <c r="C5" s="21">
-        <f>'Assumptions'!C36</f>
+        <f>'Assumptions'!C39</f>
         <v/>
       </c>
     </row>
@@ -3079,7 +3144,7 @@
         </is>
       </c>
       <c r="C24" s="16">
-        <f>'Assumptions'!C32*'Deal &amp; PPA'!C21</f>
+        <f>'Assumptions'!C35*'Deal &amp; PPA'!C21</f>
         <v/>
       </c>
     </row>
@@ -3116,7 +3181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3176,7 +3241,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Property, plant &amp; equipment</t>
+          <t>Property, plant &amp; equipment — forecast by segment</t>
         </is>
       </c>
       <c r="B3" s="9" t="n"/>
@@ -3191,783 +3256,1185 @@
       <c r="K3" s="9" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Beginning net PP&amp;E</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="n">
-        <v>46000</v>
-      </c>
-      <c r="D4" s="16">
-        <f>'Balance Sheet'!F9</f>
-        <v/>
-      </c>
-      <c r="E4" s="16">
-        <f>'Schedules'!D7</f>
-        <v/>
-      </c>
-      <c r="F4" s="16">
-        <f>'Schedules'!E7</f>
-        <v/>
-      </c>
-      <c r="G4" s="16">
-        <f>'Schedules'!F7</f>
-        <v/>
-      </c>
-      <c r="H4" s="16">
-        <f>'Schedules'!G7</f>
-        <v/>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Space</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capital expenditures</t>
+          <t xml:space="preserve">     Beginning net PP&amp;E</t>
         </is>
       </c>
       <c r="C5" s="16">
-        <f>'Assumptions'!C21*'Income Statement'!C8</f>
+        <f>'Assumptions'!C27</f>
         <v/>
       </c>
       <c r="D5" s="16">
-        <f>'Assumptions'!D21*'Income Statement'!D8</f>
+        <f>'Assumptions'!C27</f>
         <v/>
       </c>
       <c r="E5" s="16">
-        <f>'Assumptions'!E21*'Income Statement'!E8</f>
+        <f>'Schedules'!D8</f>
         <v/>
       </c>
       <c r="F5" s="16">
-        <f>'Assumptions'!F21*'Income Statement'!F8</f>
+        <f>'Schedules'!E8</f>
         <v/>
       </c>
       <c r="G5" s="16">
-        <f>'Assumptions'!G21*'Income Statement'!G8</f>
+        <f>'Schedules'!F8</f>
         <v/>
       </c>
       <c r="H5" s="16">
-        <f>'Assumptions'!H21*'Income Statement'!H8</f>
+        <f>'Schedules'!G8</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Depreciation</t>
+          <t xml:space="preserve">     (+) Capital expenditures</t>
         </is>
       </c>
       <c r="C6" s="16">
-        <f>'Schedules'!C4*'Assumptions'!C22</f>
+        <f>'Assumptions'!C21*'Segments'!C5</f>
         <v/>
       </c>
       <c r="D6" s="16">
-        <f>'Schedules'!D4*'Assumptions'!C22</f>
+        <f>'Assumptions'!D21*'Segments'!D5</f>
         <v/>
       </c>
       <c r="E6" s="16">
-        <f>'Schedules'!E4*'Assumptions'!C22</f>
+        <f>'Assumptions'!E21*'Segments'!E5</f>
         <v/>
       </c>
       <c r="F6" s="16">
-        <f>'Schedules'!F4*'Assumptions'!C22</f>
+        <f>'Assumptions'!F21*'Segments'!F5</f>
         <v/>
       </c>
       <c r="G6" s="16">
-        <f>'Schedules'!G4*'Assumptions'!C22</f>
+        <f>'Assumptions'!G21*'Segments'!G5</f>
         <v/>
       </c>
       <c r="H6" s="16">
-        <f>'Schedules'!H4*'Assumptions'!C22</f>
+        <f>'Assumptions'!H21*'Segments'!H5</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ending net PP&amp;E</t>
-        </is>
-      </c>
-      <c r="C7" s="17" t="n">
-        <v>46000</v>
-      </c>
-      <c r="D7" s="17">
-        <f>'Schedules'!D4+'Schedules'!D5-'Schedules'!D6</f>
-        <v/>
-      </c>
-      <c r="E7" s="17">
-        <f>'Schedules'!E4+'Schedules'!E5-'Schedules'!E6</f>
-        <v/>
-      </c>
-      <c r="F7" s="17">
-        <f>'Schedules'!F4+'Schedules'!F5-'Schedules'!F6</f>
-        <v/>
-      </c>
-      <c r="G7" s="17">
-        <f>'Schedules'!G4+'Schedules'!G5-'Schedules'!G6</f>
-        <v/>
-      </c>
-      <c r="H7" s="17">
-        <f>'Schedules'!H4+'Schedules'!H5-'Schedules'!H6</f>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     (−) Depreciation</t>
+        </is>
+      </c>
+      <c r="C7" s="16">
+        <f>'Schedules'!C5*'Assumptions'!C24</f>
+        <v/>
+      </c>
+      <c r="D7" s="16">
+        <f>'Schedules'!D5*'Assumptions'!C24</f>
+        <v/>
+      </c>
+      <c r="E7" s="16">
+        <f>'Schedules'!E5*'Assumptions'!C24</f>
+        <v/>
+      </c>
+      <c r="F7" s="16">
+        <f>'Schedules'!F5*'Assumptions'!C24</f>
+        <v/>
+      </c>
+      <c r="G7" s="16">
+        <f>'Schedules'!G5*'Assumptions'!C24</f>
+        <v/>
+      </c>
+      <c r="H7" s="16">
+        <f>'Schedules'!H5*'Assumptions'!C24</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Acquired intangibles &amp; deferred tax</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Ending net PP&amp;E</t>
+        </is>
+      </c>
+      <c r="C8" s="17">
+        <f>'Schedules'!C5</f>
+        <v/>
+      </c>
+      <c r="D8" s="17">
+        <f>'Schedules'!D5+'Schedules'!D6-'Schedules'!D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="17">
+        <f>'Schedules'!E5+'Schedules'!E6-'Schedules'!E7</f>
+        <v/>
+      </c>
+      <c r="F8" s="17">
+        <f>'Schedules'!F5+'Schedules'!F6-'Schedules'!F7</f>
+        <v/>
+      </c>
+      <c r="G8" s="17">
+        <f>'Schedules'!G5+'Schedules'!G6-'Schedules'!G7</f>
+        <v/>
+      </c>
+      <c r="H8" s="17">
+        <f>'Schedules'!H5+'Schedules'!H6-'Schedules'!H7</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Beginning intangibles, net</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="16">
-        <f>'Deal &amp; PPA'!C21</f>
-        <v/>
-      </c>
-      <c r="E9" s="16">
-        <f>'Schedules'!D11</f>
-        <v/>
-      </c>
-      <c r="F9" s="16">
-        <f>'Schedules'!E11</f>
-        <v/>
-      </c>
-      <c r="G9" s="16">
-        <f>'Schedules'!F11</f>
-        <v/>
-      </c>
-      <c r="H9" s="16">
-        <f>'Schedules'!G11</f>
-        <v/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Starlink</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Amortization</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>0</v>
+          <t xml:space="preserve">     Beginning net PP&amp;E</t>
+        </is>
+      </c>
+      <c r="C10" s="16">
+        <f>'Balance Sheet'!F9-'Assumptions'!C27-'Assumptions'!C28</f>
+        <v/>
       </c>
       <c r="D10" s="16">
-        <f>MIN('Schedules'!D9,'Deal &amp; PPA'!C22)</f>
+        <f>'Balance Sheet'!F9-'Assumptions'!C27-'Assumptions'!C28</f>
         <v/>
       </c>
       <c r="E10" s="16">
-        <f>MIN('Schedules'!E9,'Deal &amp; PPA'!C22)</f>
+        <f>'Schedules'!D13</f>
         <v/>
       </c>
       <c r="F10" s="16">
-        <f>MIN('Schedules'!F9,'Deal &amp; PPA'!C22)</f>
+        <f>'Schedules'!E13</f>
         <v/>
       </c>
       <c r="G10" s="16">
-        <f>MIN('Schedules'!G9,'Deal &amp; PPA'!C22)</f>
+        <f>'Schedules'!F13</f>
         <v/>
       </c>
       <c r="H10" s="16">
-        <f>MIN('Schedules'!H9,'Deal &amp; PPA'!C22)</f>
+        <f>'Schedules'!G13</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ending intangibles, net</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="17">
-        <f>'Schedules'!D9-'Schedules'!D10</f>
-        <v/>
-      </c>
-      <c r="E11" s="17">
-        <f>'Schedules'!E9-'Schedules'!E10</f>
-        <v/>
-      </c>
-      <c r="F11" s="17">
-        <f>'Schedules'!F9-'Schedules'!F10</f>
-        <v/>
-      </c>
-      <c r="G11" s="17">
-        <f>'Schedules'!G9-'Schedules'!G10</f>
-        <v/>
-      </c>
-      <c r="H11" s="17">
-        <f>'Schedules'!H9-'Schedules'!H10</f>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     (+) Capital expenditures</t>
+        </is>
+      </c>
+      <c r="C11" s="16">
+        <f>'Assumptions'!C22*'Segments'!C6</f>
+        <v/>
+      </c>
+      <c r="D11" s="16">
+        <f>'Assumptions'!D22*'Segments'!D6</f>
+        <v/>
+      </c>
+      <c r="E11" s="16">
+        <f>'Assumptions'!E22*'Segments'!E6</f>
+        <v/>
+      </c>
+      <c r="F11" s="16">
+        <f>'Assumptions'!F22*'Segments'!F6</f>
+        <v/>
+      </c>
+      <c r="G11" s="16">
+        <f>'Assumptions'!G22*'Segments'!G6</f>
+        <v/>
+      </c>
+      <c r="H11" s="16">
+        <f>'Assumptions'!H22*'Segments'!H6</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Beginning deferred tax liability</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="n">
-        <v>0</v>
+          <t xml:space="preserve">     (−) Depreciation</t>
+        </is>
+      </c>
+      <c r="C12" s="16">
+        <f>'Schedules'!C10*'Assumptions'!C25</f>
+        <v/>
       </c>
       <c r="D12" s="16">
-        <f>'Deal &amp; PPA'!C24</f>
+        <f>'Schedules'!D10*'Assumptions'!C25</f>
         <v/>
       </c>
       <c r="E12" s="16">
-        <f>'Schedules'!D14</f>
+        <f>'Schedules'!E10*'Assumptions'!C25</f>
         <v/>
       </c>
       <c r="F12" s="16">
-        <f>'Schedules'!E14</f>
+        <f>'Schedules'!F10*'Assumptions'!C25</f>
         <v/>
       </c>
       <c r="G12" s="16">
-        <f>'Schedules'!F14</f>
+        <f>'Schedules'!G10*'Assumptions'!C25</f>
         <v/>
       </c>
       <c r="H12" s="16">
-        <f>'Schedules'!G14</f>
+        <f>'Schedules'!H10*'Assumptions'!C25</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Change in DTL (deferred tax benefit)</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="16">
-        <f>-'Assumptions'!C32*'Schedules'!D10</f>
-        <v/>
-      </c>
-      <c r="E13" s="16">
-        <f>-'Assumptions'!C32*'Schedules'!E10</f>
-        <v/>
-      </c>
-      <c r="F13" s="16">
-        <f>-'Assumptions'!C32*'Schedules'!F10</f>
-        <v/>
-      </c>
-      <c r="G13" s="16">
-        <f>-'Assumptions'!C32*'Schedules'!G10</f>
-        <v/>
-      </c>
-      <c r="H13" s="16">
-        <f>-'Assumptions'!C32*'Schedules'!H10</f>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Ending net PP&amp;E</t>
+        </is>
+      </c>
+      <c r="C13" s="17">
+        <f>'Schedules'!C10</f>
+        <v/>
+      </c>
+      <c r="D13" s="17">
+        <f>'Schedules'!D10+'Schedules'!D11-'Schedules'!D12</f>
+        <v/>
+      </c>
+      <c r="E13" s="17">
+        <f>'Schedules'!E10+'Schedules'!E11-'Schedules'!E12</f>
+        <v/>
+      </c>
+      <c r="F13" s="17">
+        <f>'Schedules'!F10+'Schedules'!F11-'Schedules'!F12</f>
+        <v/>
+      </c>
+      <c r="G13" s="17">
+        <f>'Schedules'!G10+'Schedules'!G11-'Schedules'!G12</f>
+        <v/>
+      </c>
+      <c r="H13" s="17">
+        <f>'Schedules'!H10+'Schedules'!H11-'Schedules'!H12</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ending deferred tax liability</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="17">
-        <f>'Schedules'!D12+'Schedules'!D13</f>
-        <v/>
-      </c>
-      <c r="E14" s="17">
-        <f>'Schedules'!E12+'Schedules'!E13</f>
-        <v/>
-      </c>
-      <c r="F14" s="17">
-        <f>'Schedules'!F12+'Schedules'!F13</f>
-        <v/>
-      </c>
-      <c r="G14" s="17">
-        <f>'Schedules'!G12+'Schedules'!G13</f>
-        <v/>
-      </c>
-      <c r="H14" s="17">
-        <f>'Schedules'!H12+'Schedules'!H13</f>
-        <v/>
+          <t xml:space="preserve">  xAI-Cursor</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Debt &amp; spectrum obligation</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="9" t="n"/>
-      <c r="I15" s="9" t="n"/>
-      <c r="J15" s="9" t="n"/>
-      <c r="K15" s="9" t="n"/>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Beginning net PP&amp;E</t>
+        </is>
+      </c>
+      <c r="C15" s="16">
+        <f>'Assumptions'!C28</f>
+        <v/>
+      </c>
+      <c r="D15" s="16">
+        <f>'Assumptions'!C28</f>
+        <v/>
+      </c>
+      <c r="E15" s="16">
+        <f>'Schedules'!D18</f>
+        <v/>
+      </c>
+      <c r="F15" s="16">
+        <f>'Schedules'!E18</f>
+        <v/>
+      </c>
+      <c r="G15" s="16">
+        <f>'Schedules'!F18</f>
+        <v/>
+      </c>
+      <c r="H15" s="16">
+        <f>'Schedules'!G18</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Beginning long-term debt</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="n">
-        <v>12000</v>
+          <t xml:space="preserve">     (+) Capital expenditures</t>
+        </is>
+      </c>
+      <c r="C16" s="16">
+        <f>'Assumptions'!C23*'Segments'!C9</f>
+        <v/>
       </c>
       <c r="D16" s="16">
-        <f>'Balance Sheet'!F21</f>
+        <f>'Assumptions'!D23*'Segments'!D9</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>'Schedules'!D18</f>
+        <f>'Assumptions'!E23*'Segments'!E9</f>
         <v/>
       </c>
       <c r="F16" s="16">
-        <f>'Schedules'!E18</f>
+        <f>'Assumptions'!F23*'Segments'!F9</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>'Schedules'!F18</f>
+        <f>'Assumptions'!G23*'Segments'!G9</f>
         <v/>
       </c>
       <c r="H16" s="16">
-        <f>'Schedules'!G18</f>
+        <f>'Assumptions'!H23*'Segments'!H9</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Net draws / (repayments)</t>
-        </is>
-      </c>
-      <c r="C17" s="16" t="n">
-        <v>0</v>
+          <t xml:space="preserve">     (−) Depreciation</t>
+        </is>
+      </c>
+      <c r="C17" s="16">
+        <f>'Schedules'!C15*'Assumptions'!C26</f>
+        <v/>
       </c>
       <c r="D17" s="16">
-        <f>'Assumptions'!D27</f>
+        <f>'Schedules'!D15*'Assumptions'!C26</f>
         <v/>
       </c>
       <c r="E17" s="16">
-        <f>'Assumptions'!E27</f>
+        <f>'Schedules'!E15*'Assumptions'!C26</f>
         <v/>
       </c>
       <c r="F17" s="16">
-        <f>'Assumptions'!F27</f>
+        <f>'Schedules'!F15*'Assumptions'!C26</f>
         <v/>
       </c>
       <c r="G17" s="16">
-        <f>'Assumptions'!G27</f>
+        <f>'Schedules'!G15*'Assumptions'!C26</f>
         <v/>
       </c>
       <c r="H17" s="16">
-        <f>'Assumptions'!H27</f>
+        <f>'Schedules'!H15*'Assumptions'!C26</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Ending long-term debt</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="n">
-        <v>12000</v>
+          <t xml:space="preserve">     Ending net PP&amp;E</t>
+        </is>
+      </c>
+      <c r="C18" s="17">
+        <f>'Schedules'!C15</f>
+        <v/>
       </c>
       <c r="D18" s="17">
-        <f>'Schedules'!D16+'Schedules'!D17</f>
+        <f>'Schedules'!D15+'Schedules'!D16-'Schedules'!D17</f>
         <v/>
       </c>
       <c r="E18" s="17">
-        <f>'Schedules'!E16+'Schedules'!E17</f>
+        <f>'Schedules'!E15+'Schedules'!E16-'Schedules'!E17</f>
         <v/>
       </c>
       <c r="F18" s="17">
-        <f>'Schedules'!F16+'Schedules'!F17</f>
+        <f>'Schedules'!F15+'Schedules'!F16-'Schedules'!F17</f>
         <v/>
       </c>
       <c r="G18" s="17">
-        <f>'Schedules'!G16+'Schedules'!G17</f>
+        <f>'Schedules'!G15+'Schedules'!G16-'Schedules'!G17</f>
         <v/>
       </c>
       <c r="H18" s="17">
-        <f>'Schedules'!H16+'Schedules'!H17</f>
+        <f>'Schedules'!H15+'Schedules'!H16-'Schedules'!H17</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Beginning spectrum obligation</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="n">
-        <v>19600</v>
-      </c>
-      <c r="D19" s="16">
-        <f>'Balance Sheet'!F22</f>
-        <v/>
-      </c>
-      <c r="E19" s="16">
-        <f>'Schedules'!D21</f>
-        <v/>
-      </c>
-      <c r="F19" s="16">
-        <f>'Schedules'!E21</f>
-        <v/>
-      </c>
-      <c r="G19" s="16">
-        <f>'Schedules'!F21</f>
-        <v/>
-      </c>
-      <c r="H19" s="16">
-        <f>'Schedules'!G21</f>
-        <v/>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total — all segments</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Repayments</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="n">
-        <v>0</v>
+          <t xml:space="preserve">     Total beginning net PP&amp;E</t>
+        </is>
+      </c>
+      <c r="C20" s="16">
+        <f>'Schedules'!C5+'Schedules'!C10+'Schedules'!C15</f>
+        <v/>
       </c>
       <c r="D20" s="16">
-        <f>'Assumptions'!D28</f>
+        <f>'Schedules'!D5+'Schedules'!D10+'Schedules'!D15</f>
         <v/>
       </c>
       <c r="E20" s="16">
-        <f>'Assumptions'!E28</f>
+        <f>'Schedules'!E5+'Schedules'!E10+'Schedules'!E15</f>
         <v/>
       </c>
       <c r="F20" s="16">
-        <f>'Assumptions'!F28</f>
+        <f>'Schedules'!F5+'Schedules'!F10+'Schedules'!F15</f>
         <v/>
       </c>
       <c r="G20" s="16">
-        <f>'Assumptions'!G28</f>
+        <f>'Schedules'!G5+'Schedules'!G10+'Schedules'!G15</f>
         <v/>
       </c>
       <c r="H20" s="16">
-        <f>'Assumptions'!H28</f>
+        <f>'Schedules'!H5+'Schedules'!H10+'Schedules'!H15</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ending spectrum obligation</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="n">
-        <v>19600</v>
-      </c>
-      <c r="D21" s="17">
-        <f>'Schedules'!D19+'Schedules'!D20</f>
-        <v/>
-      </c>
-      <c r="E21" s="17">
-        <f>'Schedules'!E19+'Schedules'!E20</f>
-        <v/>
-      </c>
-      <c r="F21" s="17">
-        <f>'Schedules'!F19+'Schedules'!F20</f>
-        <v/>
-      </c>
-      <c r="G21" s="17">
-        <f>'Schedules'!G19+'Schedules'!G20</f>
-        <v/>
-      </c>
-      <c r="H21" s="17">
-        <f>'Schedules'!H19+'Schedules'!H20</f>
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     (+) Total capital expenditures</t>
+        </is>
+      </c>
+      <c r="C21" s="16">
+        <f>'Schedules'!C6+'Schedules'!C11+'Schedules'!C16</f>
+        <v/>
+      </c>
+      <c r="D21" s="16">
+        <f>'Schedules'!D6+'Schedules'!D11+'Schedules'!D16</f>
+        <v/>
+      </c>
+      <c r="E21" s="16">
+        <f>'Schedules'!E6+'Schedules'!E11+'Schedules'!E16</f>
+        <v/>
+      </c>
+      <c r="F21" s="16">
+        <f>'Schedules'!F6+'Schedules'!F11+'Schedules'!F16</f>
+        <v/>
+      </c>
+      <c r="G21" s="16">
+        <f>'Schedules'!G6+'Schedules'!G11+'Schedules'!G16</f>
+        <v/>
+      </c>
+      <c r="H21" s="16">
+        <f>'Schedules'!H6+'Schedules'!H11+'Schedules'!H16</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Interest expense (on beginning balances)</t>
-        </is>
-      </c>
-      <c r="C22" s="17">
-        <f>('Schedules'!C16+'Schedules'!C19)*'Assumptions'!C30</f>
-        <v/>
-      </c>
-      <c r="D22" s="17">
-        <f>('Schedules'!D16+'Schedules'!D19)*'Assumptions'!C30</f>
-        <v/>
-      </c>
-      <c r="E22" s="17">
-        <f>('Schedules'!E16+'Schedules'!E19)*'Assumptions'!C30</f>
-        <v/>
-      </c>
-      <c r="F22" s="17">
-        <f>('Schedules'!F16+'Schedules'!F19)*'Assumptions'!C30</f>
-        <v/>
-      </c>
-      <c r="G22" s="17">
-        <f>('Schedules'!G16+'Schedules'!G19)*'Assumptions'!C30</f>
-        <v/>
-      </c>
-      <c r="H22" s="17">
-        <f>('Schedules'!H16+'Schedules'!H19)*'Assumptions'!C30</f>
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     (−) Total depreciation</t>
+        </is>
+      </c>
+      <c r="C22" s="16">
+        <f>'Schedules'!C7+'Schedules'!C12+'Schedules'!C17</f>
+        <v/>
+      </c>
+      <c r="D22" s="16">
+        <f>'Schedules'!D7+'Schedules'!D12+'Schedules'!D17</f>
+        <v/>
+      </c>
+      <c r="E22" s="16">
+        <f>'Schedules'!E7+'Schedules'!E12+'Schedules'!E17</f>
+        <v/>
+      </c>
+      <c r="F22" s="16">
+        <f>'Schedules'!F7+'Schedules'!F12+'Schedules'!F17</f>
+        <v/>
+      </c>
+      <c r="G22" s="16">
+        <f>'Schedules'!G7+'Schedules'!G12+'Schedules'!G17</f>
+        <v/>
+      </c>
+      <c r="H22" s="16">
+        <f>'Schedules'!H7+'Schedules'!H12+'Schedules'!H17</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>Tax &amp; NOL carryforward</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="n"/>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="9" t="n"/>
-      <c r="H23" s="9" t="n"/>
-      <c r="I23" s="9" t="n"/>
-      <c r="J23" s="9" t="n"/>
-      <c r="K23" s="9" t="n"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Total ending net PP&amp;E</t>
+        </is>
+      </c>
+      <c r="C23" s="17">
+        <f>'Schedules'!C8+'Schedules'!C13+'Schedules'!C18</f>
+        <v/>
+      </c>
+      <c r="D23" s="17">
+        <f>'Schedules'!D8+'Schedules'!D13+'Schedules'!D18</f>
+        <v/>
+      </c>
+      <c r="E23" s="17">
+        <f>'Schedules'!E8+'Schedules'!E13+'Schedules'!E18</f>
+        <v/>
+      </c>
+      <c r="F23" s="17">
+        <f>'Schedules'!F8+'Schedules'!F13+'Schedules'!F18</f>
+        <v/>
+      </c>
+      <c r="G23" s="17">
+        <f>'Schedules'!G8+'Schedules'!G13+'Schedules'!G18</f>
+        <v/>
+      </c>
+      <c r="H23" s="17">
+        <f>'Schedules'!H8+'Schedules'!H13+'Schedules'!H18</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Pre-tax income (from IS)</t>
-        </is>
-      </c>
-      <c r="C24" s="16">
-        <f>'Income Statement'!C22</f>
-        <v/>
-      </c>
-      <c r="D24" s="16">
-        <f>'Income Statement'!D22</f>
-        <v/>
-      </c>
-      <c r="E24" s="16">
-        <f>'Income Statement'!E22</f>
-        <v/>
-      </c>
-      <c r="F24" s="16">
-        <f>'Income Statement'!F22</f>
-        <v/>
-      </c>
-      <c r="G24" s="16">
-        <f>'Income Statement'!G22</f>
-        <v/>
-      </c>
-      <c r="H24" s="16">
-        <f>'Income Statement'!H22</f>
-        <v/>
-      </c>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Acquired intangibles &amp; deferred tax</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n"/>
+      <c r="C24" s="9" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n"/>
+      <c r="I24" s="9" t="n"/>
+      <c r="J24" s="9" t="n"/>
+      <c r="K24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Taxable income (add back non-deductible amort)</t>
-        </is>
-      </c>
-      <c r="C25" s="16">
-        <f>'Schedules'!C24+'Schedules'!C10</f>
-        <v/>
+          <t xml:space="preserve">  Beginning intangibles, net</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="n">
+        <v>0</v>
       </c>
       <c r="D25" s="16">
-        <f>'Schedules'!D24+'Schedules'!D10</f>
+        <f>'Deal &amp; PPA'!C21</f>
         <v/>
       </c>
       <c r="E25" s="16">
-        <f>'Schedules'!E24+'Schedules'!E10</f>
+        <f>'Schedules'!D27</f>
         <v/>
       </c>
       <c r="F25" s="16">
-        <f>'Schedules'!F24+'Schedules'!F10</f>
+        <f>'Schedules'!E27</f>
         <v/>
       </c>
       <c r="G25" s="16">
-        <f>'Schedules'!G24+'Schedules'!G10</f>
+        <f>'Schedules'!F27</f>
         <v/>
       </c>
       <c r="H25" s="16">
-        <f>'Schedules'!H24+'Schedules'!H10</f>
+        <f>'Schedules'!G27</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Beginning NOL balance</t>
-        </is>
-      </c>
-      <c r="C26" s="16">
-        <f>'Assumptions'!C33</f>
-        <v/>
+          <t xml:space="preserve">  Amortization</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="n">
+        <v>0</v>
       </c>
       <c r="D26" s="16">
-        <f>'Schedules'!C29</f>
+        <f>MIN('Schedules'!D25,'Deal &amp; PPA'!C22)</f>
         <v/>
       </c>
       <c r="E26" s="16">
-        <f>'Schedules'!D29</f>
+        <f>MIN('Schedules'!E25,'Deal &amp; PPA'!C22)</f>
         <v/>
       </c>
       <c r="F26" s="16">
-        <f>'Schedules'!E29</f>
+        <f>MIN('Schedules'!F25,'Deal &amp; PPA'!C22)</f>
         <v/>
       </c>
       <c r="G26" s="16">
-        <f>'Schedules'!F29</f>
+        <f>MIN('Schedules'!G25,'Deal &amp; PPA'!C22)</f>
         <v/>
       </c>
       <c r="H26" s="16">
-        <f>'Schedules'!G29</f>
+        <f>MIN('Schedules'!H25,'Deal &amp; PPA'!C22)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NOL utilised</t>
-        </is>
-      </c>
-      <c r="C27" s="16">
-        <f>MIN('Schedules'!C26,'Assumptions'!C34*MAX(0,'Schedules'!C25))</f>
-        <v/>
-      </c>
-      <c r="D27" s="16">
-        <f>MIN('Schedules'!D26,'Assumptions'!C34*MAX(0,'Schedules'!D25))</f>
-        <v/>
-      </c>
-      <c r="E27" s="16">
-        <f>MIN('Schedules'!E26,'Assumptions'!C34*MAX(0,'Schedules'!E25))</f>
-        <v/>
-      </c>
-      <c r="F27" s="16">
-        <f>MIN('Schedules'!F26,'Assumptions'!C34*MAX(0,'Schedules'!F25))</f>
-        <v/>
-      </c>
-      <c r="G27" s="16">
-        <f>MIN('Schedules'!G26,'Assumptions'!C34*MAX(0,'Schedules'!G25))</f>
-        <v/>
-      </c>
-      <c r="H27" s="16">
-        <f>MIN('Schedules'!H26,'Assumptions'!C34*MAX(0,'Schedules'!H25))</f>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ending intangibles, net</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="17">
+        <f>'Schedules'!D25-'Schedules'!D26</f>
+        <v/>
+      </c>
+      <c r="E27" s="17">
+        <f>'Schedules'!E25-'Schedules'!E26</f>
+        <v/>
+      </c>
+      <c r="F27" s="17">
+        <f>'Schedules'!F25-'Schedules'!F26</f>
+        <v/>
+      </c>
+      <c r="G27" s="17">
+        <f>'Schedules'!G25-'Schedules'!G26</f>
+        <v/>
+      </c>
+      <c r="H27" s="17">
+        <f>'Schedules'!H25-'Schedules'!H26</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  NOL generated</t>
-        </is>
-      </c>
-      <c r="C28" s="16">
-        <f>MAX(0,-'Schedules'!C25)</f>
-        <v/>
+          <t xml:space="preserve">  Beginning deferred tax liability</t>
+        </is>
+      </c>
+      <c r="C28" s="16" t="n">
+        <v>0</v>
       </c>
       <c r="D28" s="16">
-        <f>MAX(0,-'Schedules'!D25)</f>
+        <f>'Deal &amp; PPA'!C24</f>
         <v/>
       </c>
       <c r="E28" s="16">
-        <f>MAX(0,-'Schedules'!E25)</f>
+        <f>'Schedules'!D30</f>
         <v/>
       </c>
       <c r="F28" s="16">
-        <f>MAX(0,-'Schedules'!F25)</f>
+        <f>'Schedules'!E30</f>
         <v/>
       </c>
       <c r="G28" s="16">
-        <f>MAX(0,-'Schedules'!G25)</f>
+        <f>'Schedules'!F30</f>
         <v/>
       </c>
       <c r="H28" s="16">
-        <f>MAX(0,-'Schedules'!H25)</f>
+        <f>'Schedules'!G30</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Ending NOL balance</t>
-        </is>
-      </c>
-      <c r="C29" s="17">
-        <f>'Schedules'!C26-'Schedules'!C27+'Schedules'!C28</f>
-        <v/>
-      </c>
-      <c r="D29" s="17">
-        <f>'Schedules'!D26-'Schedules'!D27+'Schedules'!D28</f>
-        <v/>
-      </c>
-      <c r="E29" s="17">
-        <f>'Schedules'!E26-'Schedules'!E27+'Schedules'!E28</f>
-        <v/>
-      </c>
-      <c r="F29" s="17">
-        <f>'Schedules'!F26-'Schedules'!F27+'Schedules'!F28</f>
-        <v/>
-      </c>
-      <c r="G29" s="17">
-        <f>'Schedules'!G26-'Schedules'!G27+'Schedules'!G28</f>
-        <v/>
-      </c>
-      <c r="H29" s="17">
-        <f>'Schedules'!H26-'Schedules'!H27+'Schedules'!H28</f>
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Change in DTL (deferred tax benefit)</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="16">
+        <f>-'Assumptions'!C35*'Schedules'!D26</f>
+        <v/>
+      </c>
+      <c r="E29" s="16">
+        <f>-'Assumptions'!C35*'Schedules'!E26</f>
+        <v/>
+      </c>
+      <c r="F29" s="16">
+        <f>-'Assumptions'!C35*'Schedules'!F26</f>
+        <v/>
+      </c>
+      <c r="G29" s="16">
+        <f>-'Assumptions'!C35*'Schedules'!G26</f>
+        <v/>
+      </c>
+      <c r="H29" s="16">
+        <f>-'Assumptions'!C35*'Schedules'!H26</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Ending deferred tax liability</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="17">
+        <f>'Schedules'!D28+'Schedules'!D29</f>
+        <v/>
+      </c>
+      <c r="E30" s="17">
+        <f>'Schedules'!E28+'Schedules'!E29</f>
+        <v/>
+      </c>
+      <c r="F30" s="17">
+        <f>'Schedules'!F28+'Schedules'!F29</f>
+        <v/>
+      </c>
+      <c r="G30" s="17">
+        <f>'Schedules'!G28+'Schedules'!G29</f>
+        <v/>
+      </c>
+      <c r="H30" s="17">
+        <f>'Schedules'!H28+'Schedules'!H29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Debt &amp; spectrum obligation</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="n"/>
+      <c r="C31" s="9" t="n"/>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n"/>
+      <c r="I31" s="9" t="n"/>
+      <c r="J31" s="9" t="n"/>
+      <c r="K31" s="9" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Beginning long-term debt</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D32" s="16">
+        <f>'Balance Sheet'!F21</f>
+        <v/>
+      </c>
+      <c r="E32" s="16">
+        <f>'Schedules'!D34</f>
+        <v/>
+      </c>
+      <c r="F32" s="16">
+        <f>'Schedules'!E34</f>
+        <v/>
+      </c>
+      <c r="G32" s="16">
+        <f>'Schedules'!F34</f>
+        <v/>
+      </c>
+      <c r="H32" s="16">
+        <f>'Schedules'!G34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Net draws / (repayments)</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="16">
+        <f>'Assumptions'!D30</f>
+        <v/>
+      </c>
+      <c r="E33" s="16">
+        <f>'Assumptions'!E30</f>
+        <v/>
+      </c>
+      <c r="F33" s="16">
+        <f>'Assumptions'!F30</f>
+        <v/>
+      </c>
+      <c r="G33" s="16">
+        <f>'Assumptions'!G30</f>
+        <v/>
+      </c>
+      <c r="H33" s="16">
+        <f>'Assumptions'!H30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ending long-term debt</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D34" s="17">
+        <f>'Schedules'!D32+'Schedules'!D33</f>
+        <v/>
+      </c>
+      <c r="E34" s="17">
+        <f>'Schedules'!E32+'Schedules'!E33</f>
+        <v/>
+      </c>
+      <c r="F34" s="17">
+        <f>'Schedules'!F32+'Schedules'!F33</f>
+        <v/>
+      </c>
+      <c r="G34" s="17">
+        <f>'Schedules'!G32+'Schedules'!G33</f>
+        <v/>
+      </c>
+      <c r="H34" s="17">
+        <f>'Schedules'!H32+'Schedules'!H33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Beginning spectrum obligation</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D35" s="16">
+        <f>'Balance Sheet'!F22</f>
+        <v/>
+      </c>
+      <c r="E35" s="16">
+        <f>'Schedules'!D37</f>
+        <v/>
+      </c>
+      <c r="F35" s="16">
+        <f>'Schedules'!E37</f>
+        <v/>
+      </c>
+      <c r="G35" s="16">
+        <f>'Schedules'!F37</f>
+        <v/>
+      </c>
+      <c r="H35" s="16">
+        <f>'Schedules'!G37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Repayments</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="16">
+        <f>'Assumptions'!D31</f>
+        <v/>
+      </c>
+      <c r="E36" s="16">
+        <f>'Assumptions'!E31</f>
+        <v/>
+      </c>
+      <c r="F36" s="16">
+        <f>'Assumptions'!F31</f>
+        <v/>
+      </c>
+      <c r="G36" s="16">
+        <f>'Assumptions'!G31</f>
+        <v/>
+      </c>
+      <c r="H36" s="16">
+        <f>'Assumptions'!H31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ending spectrum obligation</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D37" s="17">
+        <f>'Schedules'!D35+'Schedules'!D36</f>
+        <v/>
+      </c>
+      <c r="E37" s="17">
+        <f>'Schedules'!E35+'Schedules'!E36</f>
+        <v/>
+      </c>
+      <c r="F37" s="17">
+        <f>'Schedules'!F35+'Schedules'!F36</f>
+        <v/>
+      </c>
+      <c r="G37" s="17">
+        <f>'Schedules'!G35+'Schedules'!G36</f>
+        <v/>
+      </c>
+      <c r="H37" s="17">
+        <f>'Schedules'!H35+'Schedules'!H36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Interest expense (on beginning balances)</t>
+        </is>
+      </c>
+      <c r="C38" s="17">
+        <f>('Schedules'!C32+'Schedules'!C35)*'Assumptions'!C33</f>
+        <v/>
+      </c>
+      <c r="D38" s="17">
+        <f>('Schedules'!D32+'Schedules'!D35)*'Assumptions'!C33</f>
+        <v/>
+      </c>
+      <c r="E38" s="17">
+        <f>('Schedules'!E32+'Schedules'!E35)*'Assumptions'!C33</f>
+        <v/>
+      </c>
+      <c r="F38" s="17">
+        <f>('Schedules'!F32+'Schedules'!F35)*'Assumptions'!C33</f>
+        <v/>
+      </c>
+      <c r="G38" s="17">
+        <f>('Schedules'!G32+'Schedules'!G35)*'Assumptions'!C33</f>
+        <v/>
+      </c>
+      <c r="H38" s="17">
+        <f>('Schedules'!H32+'Schedules'!H35)*'Assumptions'!C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>Tax &amp; NOL carryforward</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="n"/>
+      <c r="C39" s="9" t="n"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" s="9" t="n"/>
+      <c r="J39" s="9" t="n"/>
+      <c r="K39" s="9" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Pre-tax income (from IS)</t>
+        </is>
+      </c>
+      <c r="C40" s="16">
+        <f>'Income Statement'!C22</f>
+        <v/>
+      </c>
+      <c r="D40" s="16">
+        <f>'Income Statement'!D22</f>
+        <v/>
+      </c>
+      <c r="E40" s="16">
+        <f>'Income Statement'!E22</f>
+        <v/>
+      </c>
+      <c r="F40" s="16">
+        <f>'Income Statement'!F22</f>
+        <v/>
+      </c>
+      <c r="G40" s="16">
+        <f>'Income Statement'!G22</f>
+        <v/>
+      </c>
+      <c r="H40" s="16">
+        <f>'Income Statement'!H22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Taxable income (add back non-deductible amort)</t>
+        </is>
+      </c>
+      <c r="C41" s="16">
+        <f>'Schedules'!C40+'Schedules'!C26</f>
+        <v/>
+      </c>
+      <c r="D41" s="16">
+        <f>'Schedules'!D40+'Schedules'!D26</f>
+        <v/>
+      </c>
+      <c r="E41" s="16">
+        <f>'Schedules'!E40+'Schedules'!E26</f>
+        <v/>
+      </c>
+      <c r="F41" s="16">
+        <f>'Schedules'!F40+'Schedules'!F26</f>
+        <v/>
+      </c>
+      <c r="G41" s="16">
+        <f>'Schedules'!G40+'Schedules'!G26</f>
+        <v/>
+      </c>
+      <c r="H41" s="16">
+        <f>'Schedules'!H40+'Schedules'!H26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Beginning NOL balance</t>
+        </is>
+      </c>
+      <c r="C42" s="16">
+        <f>'Assumptions'!C36</f>
+        <v/>
+      </c>
+      <c r="D42" s="16">
+        <f>'Schedules'!C45</f>
+        <v/>
+      </c>
+      <c r="E42" s="16">
+        <f>'Schedules'!D45</f>
+        <v/>
+      </c>
+      <c r="F42" s="16">
+        <f>'Schedules'!E45</f>
+        <v/>
+      </c>
+      <c r="G42" s="16">
+        <f>'Schedules'!F45</f>
+        <v/>
+      </c>
+      <c r="H42" s="16">
+        <f>'Schedules'!G45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOL utilised</t>
+        </is>
+      </c>
+      <c r="C43" s="16">
+        <f>MIN('Schedules'!C42,'Assumptions'!C37*MAX(0,'Schedules'!C41))</f>
+        <v/>
+      </c>
+      <c r="D43" s="16">
+        <f>MIN('Schedules'!D42,'Assumptions'!C37*MAX(0,'Schedules'!D41))</f>
+        <v/>
+      </c>
+      <c r="E43" s="16">
+        <f>MIN('Schedules'!E42,'Assumptions'!C37*MAX(0,'Schedules'!E41))</f>
+        <v/>
+      </c>
+      <c r="F43" s="16">
+        <f>MIN('Schedules'!F42,'Assumptions'!C37*MAX(0,'Schedules'!F41))</f>
+        <v/>
+      </c>
+      <c r="G43" s="16">
+        <f>MIN('Schedules'!G42,'Assumptions'!C37*MAX(0,'Schedules'!G41))</f>
+        <v/>
+      </c>
+      <c r="H43" s="16">
+        <f>MIN('Schedules'!H42,'Assumptions'!C37*MAX(0,'Schedules'!H41))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOL generated</t>
+        </is>
+      </c>
+      <c r="C44" s="16">
+        <f>MAX(0,-'Schedules'!C41)</f>
+        <v/>
+      </c>
+      <c r="D44" s="16">
+        <f>MAX(0,-'Schedules'!D41)</f>
+        <v/>
+      </c>
+      <c r="E44" s="16">
+        <f>MAX(0,-'Schedules'!E41)</f>
+        <v/>
+      </c>
+      <c r="F44" s="16">
+        <f>MAX(0,-'Schedules'!F41)</f>
+        <v/>
+      </c>
+      <c r="G44" s="16">
+        <f>MAX(0,-'Schedules'!G41)</f>
+        <v/>
+      </c>
+      <c r="H44" s="16">
+        <f>MAX(0,-'Schedules'!H41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ending NOL balance</t>
+        </is>
+      </c>
+      <c r="C45" s="17">
+        <f>'Schedules'!C42-'Schedules'!C43+'Schedules'!C44</f>
+        <v/>
+      </c>
+      <c r="D45" s="17">
+        <f>'Schedules'!D42-'Schedules'!D43+'Schedules'!D44</f>
+        <v/>
+      </c>
+      <c r="E45" s="17">
+        <f>'Schedules'!E42-'Schedules'!E43+'Schedules'!E44</f>
+        <v/>
+      </c>
+      <c r="F45" s="17">
+        <f>'Schedules'!F42-'Schedules'!F43+'Schedules'!F44</f>
+        <v/>
+      </c>
+      <c r="G45" s="17">
+        <f>'Schedules'!G42-'Schedules'!G43+'Schedules'!G44</f>
+        <v/>
+      </c>
+      <c r="H45" s="17">
+        <f>'Schedules'!H42-'Schedules'!H43+'Schedules'!H44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Current income tax</t>
         </is>
       </c>
-      <c r="C30" s="17">
-        <f>'Assumptions'!C32*MAX(0,'Schedules'!C25-'Schedules'!C27)</f>
-        <v/>
-      </c>
-      <c r="D30" s="17">
-        <f>'Assumptions'!C32*MAX(0,'Schedules'!D25-'Schedules'!D27)</f>
-        <v/>
-      </c>
-      <c r="E30" s="17">
-        <f>'Assumptions'!C32*MAX(0,'Schedules'!E25-'Schedules'!E27)</f>
-        <v/>
-      </c>
-      <c r="F30" s="17">
-        <f>'Assumptions'!C32*MAX(0,'Schedules'!F25-'Schedules'!F27)</f>
-        <v/>
-      </c>
-      <c r="G30" s="17">
-        <f>'Assumptions'!C32*MAX(0,'Schedules'!G25-'Schedules'!G27)</f>
-        <v/>
-      </c>
-      <c r="H30" s="17">
-        <f>'Assumptions'!C32*MAX(0,'Schedules'!H25-'Schedules'!H27)</f>
+      <c r="C46" s="17">
+        <f>'Assumptions'!C35*MAX(0,'Schedules'!C41-'Schedules'!C43)</f>
+        <v/>
+      </c>
+      <c r="D46" s="17">
+        <f>'Assumptions'!C35*MAX(0,'Schedules'!D41-'Schedules'!D43)</f>
+        <v/>
+      </c>
+      <c r="E46" s="17">
+        <f>'Assumptions'!C35*MAX(0,'Schedules'!E41-'Schedules'!E43)</f>
+        <v/>
+      </c>
+      <c r="F46" s="17">
+        <f>'Assumptions'!C35*MAX(0,'Schedules'!F41-'Schedules'!F43)</f>
+        <v/>
+      </c>
+      <c r="G46" s="17">
+        <f>'Assumptions'!C35*MAX(0,'Schedules'!G41-'Schedules'!G43)</f>
+        <v/>
+      </c>
+      <c r="H46" s="17">
+        <f>'Assumptions'!C35*MAX(0,'Schedules'!H41-'Schedules'!H43)</f>
         <v/>
       </c>
     </row>
@@ -4383,27 +4850,27 @@
         </is>
       </c>
       <c r="C16" s="16">
-        <f>'Schedules'!C6</f>
+        <f>'Schedules'!C22</f>
         <v/>
       </c>
       <c r="D16" s="16">
-        <f>'Schedules'!D6</f>
+        <f>'Schedules'!D22</f>
         <v/>
       </c>
       <c r="E16" s="16">
-        <f>'Schedules'!E6</f>
+        <f>'Schedules'!E22</f>
         <v/>
       </c>
       <c r="F16" s="16">
-        <f>'Schedules'!F6</f>
+        <f>'Schedules'!F22</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>'Schedules'!G6</f>
+        <f>'Schedules'!G22</f>
         <v/>
       </c>
       <c r="H16" s="16">
-        <f>'Schedules'!H6</f>
+        <f>'Schedules'!H22</f>
         <v/>
       </c>
     </row>
@@ -4414,27 +4881,27 @@
         </is>
       </c>
       <c r="C17" s="16">
-        <f>'Schedules'!C10</f>
+        <f>'Schedules'!C26</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>'Schedules'!D10</f>
+        <f>'Schedules'!D26</f>
         <v/>
       </c>
       <c r="E17" s="16">
-        <f>'Schedules'!E10</f>
+        <f>'Schedules'!E26</f>
         <v/>
       </c>
       <c r="F17" s="16">
-        <f>'Schedules'!F10</f>
+        <f>'Schedules'!F26</f>
         <v/>
       </c>
       <c r="G17" s="16">
-        <f>'Schedules'!G10</f>
+        <f>'Schedules'!G26</f>
         <v/>
       </c>
       <c r="H17" s="16">
-        <f>'Schedules'!H10</f>
+        <f>'Schedules'!H26</f>
         <v/>
       </c>
     </row>
@@ -4507,27 +4974,27 @@
         </is>
       </c>
       <c r="C20" s="16">
-        <f>-'Schedules'!C22</f>
+        <f>-'Schedules'!C38</f>
         <v/>
       </c>
       <c r="D20" s="16">
-        <f>-'Schedules'!D22</f>
+        <f>-'Schedules'!D38</f>
         <v/>
       </c>
       <c r="E20" s="16">
-        <f>-'Schedules'!E22</f>
+        <f>-'Schedules'!E38</f>
         <v/>
       </c>
       <c r="F20" s="16">
-        <f>-'Schedules'!F22</f>
+        <f>-'Schedules'!F38</f>
         <v/>
       </c>
       <c r="G20" s="16">
-        <f>-'Schedules'!G22</f>
+        <f>-'Schedules'!G38</f>
         <v/>
       </c>
       <c r="H20" s="16">
-        <f>-'Schedules'!H22</f>
+        <f>-'Schedules'!H38</f>
         <v/>
       </c>
     </row>
@@ -4538,27 +5005,27 @@
         </is>
       </c>
       <c r="C21" s="16">
-        <f>12000*'Assumptions'!C31</f>
+        <f>12000*'Assumptions'!C34</f>
         <v/>
       </c>
       <c r="D21" s="16">
-        <f>'Balance Sheet'!F4*'Assumptions'!C31</f>
+        <f>'Balance Sheet'!F4*'Assumptions'!C34</f>
         <v/>
       </c>
       <c r="E21" s="16">
-        <f>'Balance Sheet'!G4*'Assumptions'!C31</f>
+        <f>'Balance Sheet'!G4*'Assumptions'!C34</f>
         <v/>
       </c>
       <c r="F21" s="16">
-        <f>'Balance Sheet'!H4*'Assumptions'!C31</f>
+        <f>'Balance Sheet'!H4*'Assumptions'!C34</f>
         <v/>
       </c>
       <c r="G21" s="16">
-        <f>'Balance Sheet'!I4*'Assumptions'!C31</f>
+        <f>'Balance Sheet'!I4*'Assumptions'!C34</f>
         <v/>
       </c>
       <c r="H21" s="16">
-        <f>'Balance Sheet'!J4*'Assumptions'!C31</f>
+        <f>'Balance Sheet'!J4*'Assumptions'!C34</f>
         <v/>
       </c>
     </row>
@@ -4600,27 +5067,27 @@
         </is>
       </c>
       <c r="C23" s="16">
-        <f>-'Schedules'!C30</f>
+        <f>-'Schedules'!C46</f>
         <v/>
       </c>
       <c r="D23" s="16">
-        <f>-'Schedules'!D30</f>
+        <f>-'Schedules'!D46</f>
         <v/>
       </c>
       <c r="E23" s="16">
-        <f>-'Schedules'!E30</f>
+        <f>-'Schedules'!E46</f>
         <v/>
       </c>
       <c r="F23" s="16">
-        <f>-'Schedules'!F30</f>
+        <f>-'Schedules'!F46</f>
         <v/>
       </c>
       <c r="G23" s="16">
-        <f>-'Schedules'!G30</f>
+        <f>-'Schedules'!G46</f>
         <v/>
       </c>
       <c r="H23" s="16">
-        <f>-'Schedules'!H30</f>
+        <f>-'Schedules'!H46</f>
         <v/>
       </c>
     </row>
@@ -4631,27 +5098,27 @@
         </is>
       </c>
       <c r="C24" s="16">
-        <f>-'Schedules'!C13</f>
+        <f>-'Schedules'!C29</f>
         <v/>
       </c>
       <c r="D24" s="16">
-        <f>-'Schedules'!D13</f>
+        <f>-'Schedules'!D29</f>
         <v/>
       </c>
       <c r="E24" s="16">
-        <f>-'Schedules'!E13</f>
+        <f>-'Schedules'!E29</f>
         <v/>
       </c>
       <c r="F24" s="16">
-        <f>-'Schedules'!F13</f>
+        <f>-'Schedules'!F29</f>
         <v/>
       </c>
       <c r="G24" s="16">
-        <f>-'Schedules'!G13</f>
+        <f>-'Schedules'!G29</f>
         <v/>
       </c>
       <c r="H24" s="16">
-        <f>-'Schedules'!H13</f>
+        <f>-'Schedules'!H29</f>
         <v/>
       </c>
     </row>
@@ -4724,27 +5191,27 @@
         </is>
       </c>
       <c r="C27" s="23">
-        <f>'Assumptions'!C35+'Deal &amp; PPA'!C6</f>
+        <f>'Assumptions'!C38+'Deal &amp; PPA'!C6</f>
         <v/>
       </c>
       <c r="D27" s="23">
-        <f>'Assumptions'!C35+'Deal &amp; PPA'!C6</f>
+        <f>'Assumptions'!C38+'Deal &amp; PPA'!C6</f>
         <v/>
       </c>
       <c r="E27" s="23">
-        <f>'Assumptions'!C35+'Deal &amp; PPA'!C6</f>
+        <f>'Assumptions'!C38+'Deal &amp; PPA'!C6</f>
         <v/>
       </c>
       <c r="F27" s="23">
-        <f>'Assumptions'!C35+'Deal &amp; PPA'!C6</f>
+        <f>'Assumptions'!C38+'Deal &amp; PPA'!C6</f>
         <v/>
       </c>
       <c r="G27" s="23">
-        <f>'Assumptions'!C35+'Deal &amp; PPA'!C6</f>
+        <f>'Assumptions'!C38+'Deal &amp; PPA'!C6</f>
         <v/>
       </c>
       <c r="H27" s="23">
-        <f>'Assumptions'!C35+'Deal &amp; PPA'!C6</f>
+        <f>'Assumptions'!C38+'Deal &amp; PPA'!C6</f>
         <v/>
       </c>
     </row>
@@ -5080,23 +5547,23 @@
         <v/>
       </c>
       <c r="G5" s="16">
-        <f>'Income Statement'!D8*'Assumptions'!C38</f>
+        <f>'Income Statement'!D8*'Assumptions'!C41</f>
         <v/>
       </c>
       <c r="H5" s="16">
-        <f>'Income Statement'!E8*'Assumptions'!C38</f>
+        <f>'Income Statement'!E8*'Assumptions'!C41</f>
         <v/>
       </c>
       <c r="I5" s="16">
-        <f>'Income Statement'!F8*'Assumptions'!C38</f>
+        <f>'Income Statement'!F8*'Assumptions'!C41</f>
         <v/>
       </c>
       <c r="J5" s="16">
-        <f>'Income Statement'!G8*'Assumptions'!C38</f>
+        <f>'Income Statement'!G8*'Assumptions'!C41</f>
         <v/>
       </c>
       <c r="K5" s="16">
-        <f>'Income Statement'!H8*'Assumptions'!C38</f>
+        <f>'Income Statement'!H8*'Assumptions'!C41</f>
         <v/>
       </c>
     </row>
@@ -5120,23 +5587,23 @@
         <v/>
       </c>
       <c r="G6" s="16">
-        <f>'Income Statement'!D8*'Assumptions'!C39</f>
+        <f>'Income Statement'!D8*'Assumptions'!C42</f>
         <v/>
       </c>
       <c r="H6" s="16">
-        <f>'Income Statement'!E8*'Assumptions'!C39</f>
+        <f>'Income Statement'!E8*'Assumptions'!C42</f>
         <v/>
       </c>
       <c r="I6" s="16">
-        <f>'Income Statement'!F8*'Assumptions'!C39</f>
+        <f>'Income Statement'!F8*'Assumptions'!C42</f>
         <v/>
       </c>
       <c r="J6" s="16">
-        <f>'Income Statement'!G8*'Assumptions'!C39</f>
+        <f>'Income Statement'!G8*'Assumptions'!C42</f>
         <v/>
       </c>
       <c r="K6" s="16">
-        <f>'Income Statement'!H8*'Assumptions'!C39</f>
+        <f>'Income Statement'!H8*'Assumptions'!C42</f>
         <v/>
       </c>
     </row>
@@ -5160,23 +5627,23 @@
         <v/>
       </c>
       <c r="G7" s="16">
-        <f>'Income Statement'!D8*'Assumptions'!C40</f>
+        <f>'Income Statement'!D8*'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="H7" s="16">
-        <f>'Income Statement'!E8*'Assumptions'!C40</f>
+        <f>'Income Statement'!E8*'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="I7" s="16">
-        <f>'Income Statement'!F8*'Assumptions'!C40</f>
+        <f>'Income Statement'!F8*'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="J7" s="16">
-        <f>'Income Statement'!G8*'Assumptions'!C40</f>
+        <f>'Income Statement'!G8*'Assumptions'!C43</f>
         <v/>
       </c>
       <c r="K7" s="16">
-        <f>'Income Statement'!H8*'Assumptions'!C40</f>
+        <f>'Income Statement'!H8*'Assumptions'!C43</f>
         <v/>
       </c>
     </row>
@@ -5243,23 +5710,23 @@
         <v/>
       </c>
       <c r="G9" s="16">
-        <f>'Schedules'!D7</f>
+        <f>'Schedules'!D23</f>
         <v/>
       </c>
       <c r="H9" s="16">
-        <f>'Schedules'!E7</f>
+        <f>'Schedules'!E23</f>
         <v/>
       </c>
       <c r="I9" s="16">
-        <f>'Schedules'!F7</f>
+        <f>'Schedules'!F23</f>
         <v/>
       </c>
       <c r="J9" s="16">
-        <f>'Schedules'!G7</f>
+        <f>'Schedules'!G23</f>
         <v/>
       </c>
       <c r="K9" s="16">
-        <f>'Schedules'!H7</f>
+        <f>'Schedules'!H23</f>
         <v/>
       </c>
     </row>
@@ -5284,23 +5751,23 @@
         <v/>
       </c>
       <c r="G10" s="16">
-        <f>'Schedules'!D11</f>
+        <f>'Schedules'!D27</f>
         <v/>
       </c>
       <c r="H10" s="16">
-        <f>'Schedules'!E11</f>
+        <f>'Schedules'!E27</f>
         <v/>
       </c>
       <c r="I10" s="16">
-        <f>'Schedules'!F11</f>
+        <f>'Schedules'!F27</f>
         <v/>
       </c>
       <c r="J10" s="16">
-        <f>'Schedules'!G11</f>
+        <f>'Schedules'!G27</f>
         <v/>
       </c>
       <c r="K10" s="16">
-        <f>'Schedules'!H11</f>
+        <f>'Schedules'!H27</f>
         <v/>
       </c>
     </row>
@@ -5505,23 +5972,23 @@
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>'Income Statement'!D8*'Assumptions'!C41</f>
+        <f>'Income Statement'!D8*'Assumptions'!C44</f>
         <v/>
       </c>
       <c r="H16" s="16">
-        <f>'Income Statement'!E8*'Assumptions'!C41</f>
+        <f>'Income Statement'!E8*'Assumptions'!C44</f>
         <v/>
       </c>
       <c r="I16" s="16">
-        <f>'Income Statement'!F8*'Assumptions'!C41</f>
+        <f>'Income Statement'!F8*'Assumptions'!C44</f>
         <v/>
       </c>
       <c r="J16" s="16">
-        <f>'Income Statement'!G8*'Assumptions'!C41</f>
+        <f>'Income Statement'!G8*'Assumptions'!C44</f>
         <v/>
       </c>
       <c r="K16" s="16">
-        <f>'Income Statement'!H8*'Assumptions'!C41</f>
+        <f>'Income Statement'!H8*'Assumptions'!C44</f>
         <v/>
       </c>
     </row>
@@ -5545,23 +6012,23 @@
         <v/>
       </c>
       <c r="G17" s="16">
-        <f>'Income Statement'!D8*'Assumptions'!C42</f>
+        <f>'Income Statement'!D8*'Assumptions'!C45</f>
         <v/>
       </c>
       <c r="H17" s="16">
-        <f>'Income Statement'!E8*'Assumptions'!C42</f>
+        <f>'Income Statement'!E8*'Assumptions'!C45</f>
         <v/>
       </c>
       <c r="I17" s="16">
-        <f>'Income Statement'!F8*'Assumptions'!C42</f>
+        <f>'Income Statement'!F8*'Assumptions'!C45</f>
         <v/>
       </c>
       <c r="J17" s="16">
-        <f>'Income Statement'!G8*'Assumptions'!C42</f>
+        <f>'Income Statement'!G8*'Assumptions'!C45</f>
         <v/>
       </c>
       <c r="K17" s="16">
-        <f>'Income Statement'!H8*'Assumptions'!C42</f>
+        <f>'Income Statement'!H8*'Assumptions'!C45</f>
         <v/>
       </c>
     </row>
@@ -5585,23 +6052,23 @@
         <v/>
       </c>
       <c r="G18" s="16">
-        <f>'Income Statement'!D8*'Assumptions'!C43</f>
+        <f>'Income Statement'!D8*'Assumptions'!C46</f>
         <v/>
       </c>
       <c r="H18" s="16">
-        <f>'Income Statement'!E8*'Assumptions'!C43</f>
+        <f>'Income Statement'!E8*'Assumptions'!C46</f>
         <v/>
       </c>
       <c r="I18" s="16">
-        <f>'Income Statement'!F8*'Assumptions'!C43</f>
+        <f>'Income Statement'!F8*'Assumptions'!C46</f>
         <v/>
       </c>
       <c r="J18" s="16">
-        <f>'Income Statement'!G8*'Assumptions'!C43</f>
+        <f>'Income Statement'!G8*'Assumptions'!C46</f>
         <v/>
       </c>
       <c r="K18" s="16">
-        <f>'Income Statement'!H8*'Assumptions'!C43</f>
+        <f>'Income Statement'!H8*'Assumptions'!C46</f>
         <v/>
       </c>
     </row>
@@ -5625,23 +6092,23 @@
         <v/>
       </c>
       <c r="G19" s="16">
-        <f>'Income Statement'!D8*'Assumptions'!C44</f>
+        <f>'Income Statement'!D8*'Assumptions'!C47</f>
         <v/>
       </c>
       <c r="H19" s="16">
-        <f>'Income Statement'!E8*'Assumptions'!C44</f>
+        <f>'Income Statement'!E8*'Assumptions'!C47</f>
         <v/>
       </c>
       <c r="I19" s="16">
-        <f>'Income Statement'!F8*'Assumptions'!C44</f>
+        <f>'Income Statement'!F8*'Assumptions'!C47</f>
         <v/>
       </c>
       <c r="J19" s="16">
-        <f>'Income Statement'!G8*'Assumptions'!C44</f>
+        <f>'Income Statement'!G8*'Assumptions'!C47</f>
         <v/>
       </c>
       <c r="K19" s="16">
-        <f>'Income Statement'!H8*'Assumptions'!C44</f>
+        <f>'Income Statement'!H8*'Assumptions'!C47</f>
         <v/>
       </c>
     </row>
@@ -5708,23 +6175,23 @@
         <v/>
       </c>
       <c r="G21" s="16">
-        <f>'Schedules'!D18</f>
+        <f>'Schedules'!D34</f>
         <v/>
       </c>
       <c r="H21" s="16">
-        <f>'Schedules'!E18</f>
+        <f>'Schedules'!E34</f>
         <v/>
       </c>
       <c r="I21" s="16">
-        <f>'Schedules'!F18</f>
+        <f>'Schedules'!F34</f>
         <v/>
       </c>
       <c r="J21" s="16">
-        <f>'Schedules'!G18</f>
+        <f>'Schedules'!G34</f>
         <v/>
       </c>
       <c r="K21" s="16">
-        <f>'Schedules'!H18</f>
+        <f>'Schedules'!H34</f>
         <v/>
       </c>
     </row>
@@ -5748,23 +6215,23 @@
         <v/>
       </c>
       <c r="G22" s="16">
-        <f>'Schedules'!D21</f>
+        <f>'Schedules'!D37</f>
         <v/>
       </c>
       <c r="H22" s="16">
-        <f>'Schedules'!E21</f>
+        <f>'Schedules'!E37</f>
         <v/>
       </c>
       <c r="I22" s="16">
-        <f>'Schedules'!F21</f>
+        <f>'Schedules'!F37</f>
         <v/>
       </c>
       <c r="J22" s="16">
-        <f>'Schedules'!G21</f>
+        <f>'Schedules'!G37</f>
         <v/>
       </c>
       <c r="K22" s="16">
-        <f>'Schedules'!H21</f>
+        <f>'Schedules'!H37</f>
         <v/>
       </c>
     </row>
@@ -5829,23 +6296,23 @@
         <v/>
       </c>
       <c r="G24" s="16">
-        <f>'Schedules'!D14</f>
+        <f>'Schedules'!D30</f>
         <v/>
       </c>
       <c r="H24" s="16">
-        <f>'Schedules'!E14</f>
+        <f>'Schedules'!E30</f>
         <v/>
       </c>
       <c r="I24" s="16">
-        <f>'Schedules'!F14</f>
+        <f>'Schedules'!F30</f>
         <v/>
       </c>
       <c r="J24" s="16">
-        <f>'Schedules'!G14</f>
+        <f>'Schedules'!G30</f>
         <v/>
       </c>
       <c r="K24" s="16">
-        <f>'Schedules'!H14</f>
+        <f>'Schedules'!H30</f>
         <v/>
       </c>
     </row>
@@ -5970,23 +6437,23 @@
         <v/>
       </c>
       <c r="G28" s="16">
-        <f>'Balance Sheet'!F28+'Cash Flow'!D8+'Assumptions'!D29</f>
+        <f>'Balance Sheet'!F28+'Cash Flow'!D8+'Assumptions'!D32</f>
         <v/>
       </c>
       <c r="H28" s="16">
-        <f>'Balance Sheet'!G28+'Cash Flow'!E8+'Assumptions'!E29</f>
+        <f>'Balance Sheet'!G28+'Cash Flow'!E8+'Assumptions'!E32</f>
         <v/>
       </c>
       <c r="I28" s="16">
-        <f>'Balance Sheet'!H28+'Cash Flow'!F8+'Assumptions'!F29</f>
+        <f>'Balance Sheet'!H28+'Cash Flow'!F8+'Assumptions'!F32</f>
         <v/>
       </c>
       <c r="J28" s="16">
-        <f>'Balance Sheet'!I28+'Cash Flow'!G8+'Assumptions'!G29</f>
+        <f>'Balance Sheet'!I28+'Cash Flow'!G8+'Assumptions'!G32</f>
         <v/>
       </c>
       <c r="K28" s="16">
-        <f>'Balance Sheet'!J28+'Cash Flow'!H8+'Assumptions'!H29</f>
+        <f>'Balance Sheet'!J28+'Cash Flow'!H8+'Assumptions'!H32</f>
         <v/>
       </c>
     </row>
@@ -6285,23 +6752,23 @@
         </is>
       </c>
       <c r="D6" s="16">
-        <f>'Schedules'!D6</f>
+        <f>'Schedules'!D22</f>
         <v/>
       </c>
       <c r="E6" s="16">
-        <f>'Schedules'!E6</f>
+        <f>'Schedules'!E22</f>
         <v/>
       </c>
       <c r="F6" s="16">
-        <f>'Schedules'!F6</f>
+        <f>'Schedules'!F22</f>
         <v/>
       </c>
       <c r="G6" s="16">
-        <f>'Schedules'!G6</f>
+        <f>'Schedules'!G22</f>
         <v/>
       </c>
       <c r="H6" s="16">
-        <f>'Schedules'!H6</f>
+        <f>'Schedules'!H22</f>
         <v/>
       </c>
     </row>
@@ -6312,23 +6779,23 @@
         </is>
       </c>
       <c r="D7" s="16">
-        <f>'Schedules'!D10</f>
+        <f>'Schedules'!D26</f>
         <v/>
       </c>
       <c r="E7" s="16">
-        <f>'Schedules'!E10</f>
+        <f>'Schedules'!E26</f>
         <v/>
       </c>
       <c r="F7" s="16">
-        <f>'Schedules'!F10</f>
+        <f>'Schedules'!F26</f>
         <v/>
       </c>
       <c r="G7" s="16">
-        <f>'Schedules'!G10</f>
+        <f>'Schedules'!G26</f>
         <v/>
       </c>
       <c r="H7" s="16">
-        <f>'Schedules'!H10</f>
+        <f>'Schedules'!H26</f>
         <v/>
       </c>
     </row>
@@ -6339,23 +6806,23 @@
         </is>
       </c>
       <c r="D8" s="16">
-        <f>'Assumptions'!D26*'Income Statement'!D8</f>
+        <f>'Assumptions'!D29*'Income Statement'!D8</f>
         <v/>
       </c>
       <c r="E8" s="16">
-        <f>'Assumptions'!E26*'Income Statement'!E8</f>
+        <f>'Assumptions'!E29*'Income Statement'!E8</f>
         <v/>
       </c>
       <c r="F8" s="16">
-        <f>'Assumptions'!F26*'Income Statement'!F8</f>
+        <f>'Assumptions'!F29*'Income Statement'!F8</f>
         <v/>
       </c>
       <c r="G8" s="16">
-        <f>'Assumptions'!G26*'Income Statement'!G8</f>
+        <f>'Assumptions'!G29*'Income Statement'!G8</f>
         <v/>
       </c>
       <c r="H8" s="16">
-        <f>'Assumptions'!H26*'Income Statement'!H8</f>
+        <f>'Assumptions'!H29*'Income Statement'!H8</f>
         <v/>
       </c>
     </row>
@@ -6366,23 +6833,23 @@
         </is>
       </c>
       <c r="D9" s="16">
-        <f>'Schedules'!D13</f>
+        <f>'Schedules'!D29</f>
         <v/>
       </c>
       <c r="E9" s="16">
-        <f>'Schedules'!E13</f>
+        <f>'Schedules'!E29</f>
         <v/>
       </c>
       <c r="F9" s="16">
-        <f>'Schedules'!F13</f>
+        <f>'Schedules'!F29</f>
         <v/>
       </c>
       <c r="G9" s="16">
-        <f>'Schedules'!G13</f>
+        <f>'Schedules'!G29</f>
         <v/>
       </c>
       <c r="H9" s="16">
-        <f>'Schedules'!H13</f>
+        <f>'Schedules'!H29</f>
         <v/>
       </c>
     </row>
@@ -6653,23 +7120,23 @@
         </is>
       </c>
       <c r="D20" s="16">
-        <f>-'Schedules'!D5</f>
+        <f>-'Schedules'!D21</f>
         <v/>
       </c>
       <c r="E20" s="16">
-        <f>-'Schedules'!E5</f>
+        <f>-'Schedules'!E21</f>
         <v/>
       </c>
       <c r="F20" s="16">
-        <f>-'Schedules'!F5</f>
+        <f>-'Schedules'!F21</f>
         <v/>
       </c>
       <c r="G20" s="16">
-        <f>-'Schedules'!G5</f>
+        <f>-'Schedules'!G21</f>
         <v/>
       </c>
       <c r="H20" s="16">
-        <f>-'Schedules'!H5</f>
+        <f>-'Schedules'!H21</f>
         <v/>
       </c>
     </row>
@@ -6724,23 +7191,23 @@
         </is>
       </c>
       <c r="D23" s="16">
-        <f>'Schedules'!D17</f>
+        <f>'Schedules'!D33</f>
         <v/>
       </c>
       <c r="E23" s="16">
-        <f>'Schedules'!E17</f>
+        <f>'Schedules'!E33</f>
         <v/>
       </c>
       <c r="F23" s="16">
-        <f>'Schedules'!F17</f>
+        <f>'Schedules'!F33</f>
         <v/>
       </c>
       <c r="G23" s="16">
-        <f>'Schedules'!G17</f>
+        <f>'Schedules'!G33</f>
         <v/>
       </c>
       <c r="H23" s="16">
-        <f>'Schedules'!H17</f>
+        <f>'Schedules'!H33</f>
         <v/>
       </c>
     </row>
@@ -6751,23 +7218,23 @@
         </is>
       </c>
       <c r="D24" s="16">
-        <f>'Schedules'!D20</f>
+        <f>'Schedules'!D36</f>
         <v/>
       </c>
       <c r="E24" s="16">
-        <f>'Schedules'!E20</f>
+        <f>'Schedules'!E36</f>
         <v/>
       </c>
       <c r="F24" s="16">
-        <f>'Schedules'!F20</f>
+        <f>'Schedules'!F36</f>
         <v/>
       </c>
       <c r="G24" s="16">
-        <f>'Schedules'!G20</f>
+        <f>'Schedules'!G36</f>
         <v/>
       </c>
       <c r="H24" s="16">
-        <f>'Schedules'!H20</f>
+        <f>'Schedules'!H36</f>
         <v/>
       </c>
     </row>
@@ -6778,23 +7245,23 @@
         </is>
       </c>
       <c r="D25" s="16">
-        <f>'Assumptions'!D29</f>
+        <f>'Assumptions'!D32</f>
         <v/>
       </c>
       <c r="E25" s="16">
-        <f>'Assumptions'!E29</f>
+        <f>'Assumptions'!E32</f>
         <v/>
       </c>
       <c r="F25" s="16">
-        <f>'Assumptions'!F29</f>
+        <f>'Assumptions'!F32</f>
         <v/>
       </c>
       <c r="G25" s="16">
-        <f>'Assumptions'!G29</f>
+        <f>'Assumptions'!G32</f>
         <v/>
       </c>
       <c r="H25" s="16">
-        <f>'Assumptions'!H29</f>
+        <f>'Assumptions'!H32</f>
         <v/>
       </c>
     </row>

</xml_diff>